<commit_message>
Add August's sheet and July's remaining source files
July: the wellness banner and the two blog thumbnails, the announcement image
now a genuine PNG rather than a renamed HEIC, and the June reference kept in
HTML/ for comparison. content.xlsx and content.json move to their current
state.

August: the sheet as it stands. Its Row Data folders exist but are still
empty, so nothing else to add yet.

The generated newsletter and email files are ignored by name, so only the
reference copy in HTML/ is tracked.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/July-2026/content.xlsx
+++ b/July-2026/content.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\Newsletter\July-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E255B858-AB27-49E5-B9F6-B9494AD7FF29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{305AE437-D58D-4717-9A97-478E2861B4F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -366,7 +366,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="99">
   <si>
     <t>BIZTECH NEWSLETTER — fill in the Content column only. Leave the grey Photos Folder / Field columns alone.</t>
   </si>
@@ -593,7 +593,80 @@
     <t>Work Anniversary (This Month)</t>
   </si>
   <si>
-    <t>Tushar Avugandey -office boy	11 years
+    <t>anniversary</t>
+  </si>
+  <si>
+    <t>Employee Certifications (This Month)</t>
+  </si>
+  <si>
+    <t>Row Data/certification</t>
+  </si>
+  <si>
+    <t>employee_certification</t>
+  </si>
+  <si>
+    <t>New Openings (This Month)</t>
+  </si>
+  <si>
+    <t>Position	Experience	Opening
+SEO Executive	Fresher	1
+Business Development Executive	2+ years	2
+System Administrator	2+ years	1</t>
+  </si>
+  <si>
+    <t>new_openings_sheet</t>
+  </si>
+  <si>
+    <t>Employee Training (This Month)</t>
+  </si>
+  <si>
+    <t>Row Data/training</t>
+  </si>
+  <si>
+    <t>employee_training</t>
+  </si>
+  <si>
+    <t>Employee Workshop (This Month)</t>
+  </si>
+  <si>
+    <t>Row Data/workshop</t>
+  </si>
+  <si>
+    <t>employee_workshop</t>
+  </si>
+  <si>
+    <t>Announcement of any Events</t>
+  </si>
+  <si>
+    <t>Independence Day Celebration</t>
+  </si>
+  <si>
+    <t>Row Data/announcement</t>
+  </si>
+  <si>
+    <t>new_announcement</t>
+  </si>
+  <si>
+    <t>Marketing Highlights (Blogs, Case Studies…)</t>
+  </si>
+  <si>
+    <t>Dhaval</t>
+  </si>
+  <si>
+    <t>Row Data/marketing/blogs</t>
+  </si>
+  <si>
+    <t>marketing_highlights</t>
+  </si>
+  <si>
+    <t>Every new quarter is a reminder that progress isn't defined by where we begin, but by the choices we make every day. Let's challenge ourselves to think bigger, embrace change with confidence, and turn every opportunity into meaningful growth. Together, let's build a quarter we'll be proud to look back on.</t>
+  </si>
+  <si>
+    <t>https://www.biztechcs.com/blog/odoo-go-live-checklist-20-things-to-varify-before-cutover/
+https://www.biztechcs.com/blog/build-internal-knowledge-base-with-llm/</t>
+  </si>
+  <si>
+    <t>Tushar Avugandey 11 years
 Viral savaj	13 years
 Bhamini Prajapati 	11 years
 Dhaval Panara	10 years
@@ -626,81 +699,12 @@
 Nidhi Rajput	3 years
 Nilesh Negi	2 years</t>
   </si>
-  <si>
-    <t>anniversary</t>
-  </si>
-  <si>
-    <t>Employee Certifications (This Month)</t>
-  </si>
-  <si>
-    <t>Row Data/certification</t>
-  </si>
-  <si>
-    <t>employee_certification</t>
-  </si>
-  <si>
-    <t>New Openings (This Month)</t>
-  </si>
-  <si>
-    <t>Position	Experience	Opening
-SEO Executive	Fresher	1
-Business Development Executive	2+ years	2
-System Administrator	2+ years	1</t>
-  </si>
-  <si>
-    <t>new_openings_sheet</t>
-  </si>
-  <si>
-    <t>Employee Training (This Month)</t>
-  </si>
-  <si>
-    <t>Row Data/training</t>
-  </si>
-  <si>
-    <t>employee_training</t>
-  </si>
-  <si>
-    <t>Employee Workshop (This Month)</t>
-  </si>
-  <si>
-    <t>Row Data/workshop</t>
-  </si>
-  <si>
-    <t>employee_workshop</t>
-  </si>
-  <si>
-    <t>Announcement of any Events</t>
-  </si>
-  <si>
-    <t>Independence Day Celebration</t>
-  </si>
-  <si>
-    <t>Row Data/announcement</t>
-  </si>
-  <si>
-    <t>new_announcement</t>
-  </si>
-  <si>
-    <t>Marketing Highlights (Blogs, Case Studies…)</t>
-  </si>
-  <si>
-    <t>Dhaval</t>
-  </si>
-  <si>
-    <t>Row Data/marketing/blogs</t>
-  </si>
-  <si>
-    <t>marketing_highlights</t>
-  </si>
-  <si>
-    <t>Every new quarter is a reminder that progress isn't defined by where we begin, but by the choices we make every day. Let's challenge ourselves to think bigger, embrace change with confidence, and turn every opportunity into meaningful growth. Together, let's build a quarter we'll be proud to look back on.</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -729,6 +733,14 @@
       <sz val="9"/>
       <color rgb="FF777777"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -771,10 +783,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -788,11 +801,15 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1106,103 +1123,103 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -1268,7 +1285,7 @@
         <v>23</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>24</v>
@@ -1557,11 +1574,11 @@
         <v>52</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G29" s="3"/>
     </row>
@@ -1570,17 +1587,17 @@
         <v>15</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D30" s="3"/>
       <c r="E30" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F30" s="4" t="s">
         <v>78</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>79</v>
       </c>
       <c r="G30" s="3"/>
     </row>
@@ -1589,17 +1606,17 @@
         <v>16</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E31" s="4"/>
       <c r="F31" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G31" s="3"/>
     </row>
@@ -1608,17 +1625,17 @@
         <v>17</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F32" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>85</v>
       </c>
       <c r="G32" s="3"/>
     </row>
@@ -1627,17 +1644,17 @@
         <v>18</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F33" s="4" t="s">
         <v>87</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>88</v>
       </c>
       <c r="G33" s="3"/>
     </row>
@@ -1646,19 +1663,19 @@
         <v>19</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D34" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E34" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="F34" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>92</v>
       </c>
       <c r="G34" s="3"/>
     </row>
@@ -1667,17 +1684,19 @@
         <v>20</v>
       </c>
       <c r="B35" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="D35" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D35" s="3"/>
-      <c r="E35" s="4" t="s">
+      <c r="F35" s="4" t="s">
         <v>95</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>96</v>
       </c>
       <c r="G35" s="3"/>
     </row>
@@ -1698,7 +1717,10 @@
       <formula1>"NA"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="D35" r:id="rId1" display="https://www.biztechcs.com/blog/odoo-go-live-checklist-20-things-to-varify-before-cutover/" xr:uid="{65C958E6-4C1F-4226-9411-86BDDC7FF022}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>